<commit_message>
feat: Agregar lógica para convertir el total de combustible autorizado a letras y actualizar la gestión de combustible en PlanViajeDto
</commit_message>
<xml_diff>
--- a/src/WebApp.Web/wwwroot/Templates/PlanViajeTemplate.xlsx
+++ b/src/WebApp.Web/wwwroot/Templates/PlanViajeTemplate.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Fonagro\src\WebApp.Web\Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Fonagro\src\WebApp.Web\wwwroot\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FB5FA7D-2B87-4F32-97A3-4BAFB8D84A14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9192"/>
+    <workbookView xWindow="-20610" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PlanViajeTemplate" sheetId="3" r:id="rId1"/>
@@ -131,7 +132,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="d/m/yy"/>
@@ -431,13 +432,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -454,43 +455,30 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="20" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -501,22 +489,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -547,17 +519,35 @@
     <xf numFmtId="164" fontId="8" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="20" fontId="1" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="1" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Millares 2" xfId="2"/>
+    <cellStyle name="Millares 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -897,7 +887,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -1512,7 +1502,7 @@
       <c r="F6" s="8"/>
     </row>
     <row r="7" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A7" s="23" t="s">
+      <c r="A7" s="19" t="s">
         <v>3</v>
       </c>
       <c r="B7" s="5" t="s">
@@ -1532,38 +1522,38 @@
       <c r="F8" s="8"/>
     </row>
     <row r="9" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="37" t="s">
+      <c r="A9" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="37"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="38" t="s">
+      <c r="B9" s="44"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="45" t="s">
         <v>5</v>
       </c>
-      <c r="E9" s="38"/>
-      <c r="F9" s="15"/>
+      <c r="E9" s="45"/>
+      <c r="F9" s="8"/>
     </row>
     <row r="10" spans="1:6" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="22" t="s">
+      <c r="A10" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="57"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="22" t="s">
+      <c r="B10" s="42"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="E10" s="57"/>
+      <c r="E10" s="42"/>
     </row>
     <row r="11" spans="1:6" ht="13.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="B11" s="58"/>
-      <c r="C11" s="21"/>
-      <c r="D11" s="22" t="s">
+      <c r="B11" s="43"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="E11" s="58"/>
+      <c r="E11" s="43"/>
     </row>
     <row r="12" spans="1:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="9"/>
@@ -1574,7 +1564,7 @@
       <c r="F12" s="8"/>
     </row>
     <row r="13" spans="1:6" ht="13.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="25" t="s">
+      <c r="A13" s="7" t="s">
         <v>6</v>
       </c>
       <c r="B13" s="5"/>
@@ -1584,86 +1574,86 @@
       <c r="F13" s="5"/>
     </row>
     <row r="14" spans="1:6" ht="68.400000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="39"/>
-      <c r="B14" s="40"/>
-      <c r="C14" s="40"/>
-      <c r="D14" s="40"/>
-      <c r="E14" s="40"/>
-      <c r="F14" s="41"/>
+      <c r="A14" s="46"/>
+      <c r="B14" s="47"/>
+      <c r="C14" s="47"/>
+      <c r="D14" s="47"/>
+      <c r="E14" s="47"/>
+      <c r="F14" s="48"/>
     </row>
     <row r="15" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A15" s="30"/>
-      <c r="B15" s="31"/>
-      <c r="C15" s="31"/>
-      <c r="D15" s="31"/>
-      <c r="E15" s="31"/>
+      <c r="A15" s="4"/>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
       <c r="F15" s="5"/>
     </row>
     <row r="16" spans="1:6" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="46" t="s">
+      <c r="A16" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="B16" s="47"/>
-      <c r="C16" s="47"/>
-      <c r="D16" s="47"/>
-      <c r="E16" s="47"/>
-      <c r="F16" s="47"/>
+      <c r="B16" s="32"/>
+      <c r="C16" s="32"/>
+      <c r="D16" s="32"/>
+      <c r="E16" s="32"/>
+      <c r="F16" s="32"/>
     </row>
     <row r="17" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A17" s="48" t="s">
+      <c r="A17" s="33" t="s">
         <v>8</v>
       </c>
-      <c r="B17" s="55" t="s">
+      <c r="B17" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="C17" s="55" t="s">
+      <c r="C17" s="40" t="s">
         <v>11</v>
       </c>
-      <c r="D17" s="55" t="s">
+      <c r="D17" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="E17" s="55" t="s">
+      <c r="E17" s="40" t="s">
         <v>13</v>
       </c>
-      <c r="F17" s="56" t="s">
+      <c r="F17" s="41" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="49"/>
-      <c r="B18" s="34">
+      <c r="A18" s="34"/>
+      <c r="B18" s="25">
         <v>0</v>
       </c>
-      <c r="C18" s="34">
+      <c r="C18" s="25">
         <v>0</v>
       </c>
-      <c r="D18" s="34">
+      <c r="D18" s="25">
         <v>0</v>
       </c>
-      <c r="E18" s="34">
+      <c r="E18" s="25">
         <v>0</v>
       </c>
-      <c r="F18" s="44">
+      <c r="F18" s="29">
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="50" t="s">
+      <c r="A19" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="43">
+      <c r="B19" s="28">
         <v>0</v>
       </c>
-      <c r="C19" s="43">
+      <c r="C19" s="28">
         <v>0</v>
       </c>
-      <c r="D19" s="43">
+      <c r="D19" s="28">
         <v>0</v>
       </c>
-      <c r="E19" s="43">
+      <c r="E19" s="28">
         <v>0</v>
       </c>
-      <c r="F19" s="45">
+      <c r="F19" s="30">
         <v>0</v>
       </c>
     </row>
@@ -1687,56 +1677,56 @@
       <c r="E21" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="F21" s="19"/>
+      <c r="F21" s="12"/>
     </row>
     <row r="22" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="48" t="s">
+      <c r="A22" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="B22" s="51" t="s">
+      <c r="B22" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="C22" s="51" t="s">
+      <c r="C22" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="D22" s="51" t="s">
+      <c r="D22" s="36" t="s">
         <v>21</v>
       </c>
-      <c r="E22" s="52" t="s">
+      <c r="E22" s="37" t="s">
         <v>22</v>
       </c>
       <c r="F22"/>
     </row>
     <row r="23" spans="1:6" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="53"/>
-      <c r="B23" s="34">
+      <c r="A23" s="38"/>
+      <c r="B23" s="25">
         <v>0</v>
       </c>
-      <c r="C23" s="35">
+      <c r="C23" s="26">
         <v>0</v>
       </c>
-      <c r="D23" s="34">
+      <c r="D23" s="25">
         <v>0</v>
       </c>
-      <c r="E23" s="44">
+      <c r="E23" s="29">
         <v>0</v>
       </c>
       <c r="F23"/>
     </row>
     <row r="24" spans="1:6" ht="12.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="50" t="s">
+      <c r="A24" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="B24" s="43">
+      <c r="B24" s="28">
         <v>0</v>
       </c>
-      <c r="C24" s="54">
+      <c r="C24" s="39">
         <v>0</v>
       </c>
-      <c r="D24" s="43">
+      <c r="D24" s="28">
         <v>0</v>
       </c>
-      <c r="E24" s="45">
+      <c r="E24" s="30">
         <v>0</v>
       </c>
       <c r="F24"/>
@@ -1747,17 +1737,17 @@
       <c r="C25" s="11"/>
       <c r="D25" s="12"/>
       <c r="E25" s="12"/>
-      <c r="F25" s="19"/>
+      <c r="F25" s="12"/>
     </row>
     <row r="26" spans="1:6" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4"/>
       <c r="B26" s="5"/>
       <c r="C26" s="5"/>
       <c r="D26" s="5"/>
-      <c r="E26" s="36" t="s">
+      <c r="E26" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="F26" s="32"/>
+      <c r="F26" s="23"/>
     </row>
     <row r="27" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
@@ -1767,7 +1757,7 @@
       <c r="C27" s="8"/>
       <c r="D27" s="8"/>
       <c r="E27" s="8"/>
-      <c r="F27" s="42"/>
+      <c r="F27" s="49"/>
     </row>
     <row r="28" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A28" s="7"/>
@@ -1786,17 +1776,17 @@
       <c r="F29" s="8"/>
     </row>
     <row r="30" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A30" s="28"/>
-      <c r="C30" s="24"/>
+      <c r="A30" s="20"/>
+      <c r="C30" s="13"/>
       <c r="D30" s="8"/>
       <c r="E30" s="8"/>
       <c r="F30" s="8"/>
     </row>
     <row r="31" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A31" s="29" t="s">
+      <c r="A31" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="C31" s="14"/>
+      <c r="C31" s="7"/>
       <c r="D31" s="8"/>
       <c r="E31" s="8"/>
       <c r="F31" s="8"/>
@@ -1818,38 +1808,38 @@
       <c r="F33" s="5"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A35" s="17"/>
+      <c r="A35" s="14"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A36" s="26" t="s">
+      <c r="A36" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="D36" s="27" t="s">
+      <c r="D36" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="E36" s="17"/>
-      <c r="F36" s="17"/>
+      <c r="E36" s="14"/>
+      <c r="F36" s="14"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C38" s="16"/>
+      <c r="C38" s="13"/>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" s="13"/>
-      <c r="C46" s="16"/>
-      <c r="D46" s="27" t="s">
+      <c r="C46" s="13"/>
+      <c r="D46" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="E46" s="17"/>
-      <c r="F46" s="17"/>
+      <c r="E46" s="14"/>
+      <c r="F46" s="14"/>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A47" s="29" t="s">
+      <c r="A47" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="E47" s="33" t="s">
+      <c r="E47" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="F47" s="18"/>
+      <c r="F47" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>